<commit_message>
Add Account Name to the template, dashboard, and PDF, and document current behavior.
Keep Opportunity Name as the customer key while showing Account Name on slides, the portfolio table, and customer PDFs, and update the README so GitHub matches this workflow.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/check_back_template.xlsx
+++ b/samples/check_back_template.xlsx
@@ -460,259 +460,264 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW2"/>
+  <dimension ref="A1:AX2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="75" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>Account Name</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
           <t>Opportunity Name</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Opportunity (linked)</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>SL2</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>TCV $</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Closed on (MM/YY)</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Competitor</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Migrating from</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Migrating to</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>CSM Engagement Model (linked)</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>CSM name</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Sub #</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Sub Term</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Sub start date (MM/DD/YYYY)</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>Add-ons included or not</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>Calling Setup Assist included (Y/N)</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>Provisioned/Entitled Lic Calling</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Active Lic Calling</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>Customer org id</t>
         </is>
       </c>
-      <c r="T1" s="4" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>Notes from Calling Analytics</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>Notes from provisioned features</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>CCEP trial (Y/N)</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>(G/Y/R)</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
         <is>
           <t>TAC/BEMS</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>AAR $</t>
         </is>
       </c>
-      <c r="Z1" s="4" t="inlineStr">
+      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>Collab AE/SE</t>
         </is>
       </c>
-      <c r="AA1" s="4" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>Service lines</t>
         </is>
       </c>
-      <c r="AB1" s="4" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>Sub term (months)</t>
         </is>
       </c>
-      <c r="AC1" s="4" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>Subscription dates</t>
         </is>
       </c>
-      <c r="AD1" s="4" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>Platforms</t>
         </is>
       </c>
-      <c r="AE1" s="4" t="inlineStr">
+      <c r="AF1" s="4" t="inlineStr">
         <is>
           <t>Trend active users 90d</t>
         </is>
       </c>
-      <c r="AF1" s="4" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>Trend call volume 90d</t>
         </is>
       </c>
-      <c r="AG1" s="4" t="inlineStr">
+      <c r="AH1" s="4" t="inlineStr">
         <is>
           <t>Lic Professional (used/entitled)</t>
         </is>
       </c>
-      <c r="AH1" s="4" t="inlineStr">
+      <c r="AI1" s="4" t="inlineStr">
         <is>
           <t>Lic Standard (used/entitled)</t>
         </is>
       </c>
-      <c r="AI1" s="4" t="inlineStr">
+      <c r="AJ1" s="4" t="inlineStr">
         <is>
           <t>Lic Workspace (used/entitled)</t>
         </is>
       </c>
-      <c r="AJ1" s="4" t="inlineStr">
+      <c r="AK1" s="4" t="inlineStr">
         <is>
           <t>Active % of provisioned</t>
         </is>
       </c>
-      <c r="AK1" s="4" t="inlineStr">
+      <c r="AL1" s="4" t="inlineStr">
         <is>
           <t>External calls</t>
         </is>
       </c>
-      <c r="AL1" s="4" t="inlineStr">
+      <c r="AM1" s="4" t="inlineStr">
         <is>
           <t>Meetings usage</t>
         </is>
       </c>
-      <c r="AM1" s="4" t="inlineStr">
+      <c r="AN1" s="4" t="inlineStr">
         <is>
           <t>Messaging usage</t>
         </is>
       </c>
-      <c r="AN1" s="4" t="inlineStr">
+      <c r="AO1" s="4" t="inlineStr">
         <is>
           <t>Auto Attendant count</t>
         </is>
       </c>
-      <c r="AO1" s="4" t="inlineStr">
+      <c r="AP1" s="4" t="inlineStr">
         <is>
           <t>Hunt Groups count</t>
         </is>
       </c>
-      <c r="AP1" s="4" t="inlineStr">
+      <c r="AQ1" s="4" t="inlineStr">
         <is>
           <t>Call Queues count</t>
         </is>
       </c>
-      <c r="AQ1" s="4" t="inlineStr">
+      <c r="AR1" s="4" t="inlineStr">
         <is>
           <t>Connected-UC (Y/N)</t>
         </is>
       </c>
-      <c r="AR1" s="4" t="inlineStr">
+      <c r="AS1" s="4" t="inlineStr">
         <is>
           <t>Virtual Lines count</t>
         </is>
       </c>
-      <c r="AS1" s="4" t="inlineStr">
+      <c r="AT1" s="4" t="inlineStr">
         <is>
           <t>Data gathered by</t>
         </is>
       </c>
-      <c r="AT1" s="4" t="inlineStr">
+      <c r="AU1" s="4" t="inlineStr">
         <is>
           <t>Data gathered date</t>
         </is>
       </c>
-      <c r="AU1" s="4" t="inlineStr">
+      <c r="AV1" s="4" t="inlineStr">
         <is>
           <t>Salesforce URL</t>
         </is>
       </c>
-      <c r="AV1" s="4" t="inlineStr">
+      <c r="AW1" s="4" t="inlineStr">
         <is>
           <t>Success Portal</t>
         </is>
       </c>
-      <c r="AW1" s="4" t="inlineStr">
+      <c r="AX1" s="4" t="inlineStr">
         <is>
           <t>Recommended Actions</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="M2" s="1" t="n"/>
-      <c r="Q2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Customer Assist Queues and format dashboard numbers with commas.
Show the new feature count on the BIA slide and PDF, and display counts and license pairs as 1,200 instead of 1200.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/check_back_template.xlsx
+++ b/samples/check_back_template.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX2"/>
+  <dimension ref="A1:AY2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="75" customHeight="1">
@@ -681,35 +681,40 @@
       </c>
       <c r="AR1" s="4" t="inlineStr">
         <is>
+          <t>Customer Assist Queues count</t>
+        </is>
+      </c>
+      <c r="AS1" s="4" t="inlineStr">
+        <is>
           <t>Connected-UC (Y/N)</t>
         </is>
       </c>
-      <c r="AS1" s="4" t="inlineStr">
+      <c r="AT1" s="4" t="inlineStr">
         <is>
           <t>Virtual Lines count</t>
         </is>
       </c>
-      <c r="AT1" s="4" t="inlineStr">
+      <c r="AU1" s="4" t="inlineStr">
         <is>
           <t>Data gathered by</t>
         </is>
       </c>
-      <c r="AU1" s="4" t="inlineStr">
+      <c r="AV1" s="4" t="inlineStr">
         <is>
           <t>Data gathered date</t>
         </is>
       </c>
-      <c r="AV1" s="4" t="inlineStr">
+      <c r="AW1" s="4" t="inlineStr">
         <is>
           <t>Salesforce URL</t>
         </is>
       </c>
-      <c r="AW1" s="4" t="inlineStr">
+      <c r="AX1" s="4" t="inlineStr">
         <is>
           <t>Success Portal</t>
         </is>
       </c>
-      <c r="AX1" s="4" t="inlineStr">
+      <c r="AY1" s="4" t="inlineStr">
         <is>
           <t>Recommended Actions</t>
         </is>

</xml_diff>

<commit_message>
Map health flags to G/Y/R/U and match year-bar length on Ny.
Good/Risk/Critical/Upsell follow the new letter map, the template column is (G/Y/R/U), and Term values like 3Y set a 3-year bar.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/check_back_template.xlsx
+++ b/samples/check_back_template.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Customer Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -581,7 +581,7 @@
       </c>
       <c r="X1" s="4" t="inlineStr">
         <is>
-          <t>(G/Y/R)</t>
+          <t>(G/Y/R/U)</t>
         </is>
       </c>
       <c r="Y1" s="4" t="inlineStr">

</xml_diff>